<commit_message>
Tu dien +76 muc: do chau A, rau VN, thit ca gastro, bia Sec (446 muc)
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tudien.xlsx
+++ b/tudien.xlsx
@@ -39,7 +39,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001A7A3A"/>
+        <fgColor rgb="00B96A1E"/>
       </patternFill>
     </fill>
   </fills>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D351"/>
+  <dimension ref="A1:D447"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -8154,6 +8154,2118 @@
         </is>
       </c>
     </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>bun</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>bún</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>ryzove nudle</t>
+        </is>
+      </c>
+      <c r="D352" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="353">
+      <c r="A353" t="inlineStr">
+        <is>
+          <t>banh pho</t>
+        </is>
+      </c>
+      <c r="B353" t="inlineStr">
+        <is>
+          <t>bánh phở</t>
+        </is>
+      </c>
+      <c r="C353" t="inlineStr">
+        <is>
+          <t>pho nudle</t>
+        </is>
+      </c>
+      <c r="D353" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="354">
+      <c r="A354" t="inlineStr">
+        <is>
+          <t>pho</t>
+        </is>
+      </c>
+      <c r="B354" t="inlineStr">
+        <is>
+          <t>phở</t>
+        </is>
+      </c>
+      <c r="C354" t="inlineStr">
+        <is>
+          <t>pho</t>
+        </is>
+      </c>
+      <c r="D354" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="355">
+      <c r="A355" t="inlineStr">
+        <is>
+          <t>hu tieu</t>
+        </is>
+      </c>
+      <c r="B355" t="inlineStr">
+        <is>
+          <t>hủ tiếu</t>
+        </is>
+      </c>
+      <c r="C355" t="inlineStr">
+        <is>
+          <t>ryzove nudle</t>
+        </is>
+      </c>
+      <c r="D355" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="356">
+      <c r="A356" t="inlineStr">
+        <is>
+          <t>mi udon</t>
+        </is>
+      </c>
+      <c r="B356" t="inlineStr">
+        <is>
+          <t>mì udon</t>
+        </is>
+      </c>
+      <c r="C356" t="inlineStr">
+        <is>
+          <t>udon</t>
+        </is>
+      </c>
+      <c r="D356" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="357">
+      <c r="A357" t="inlineStr">
+        <is>
+          <t>mi soba</t>
+        </is>
+      </c>
+      <c r="B357" t="inlineStr">
+        <is>
+          <t>mì soba</t>
+        </is>
+      </c>
+      <c r="C357" t="inlineStr">
+        <is>
+          <t>soba</t>
+        </is>
+      </c>
+      <c r="D357" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="358">
+      <c r="A358" t="inlineStr">
+        <is>
+          <t>mi ramen</t>
+        </is>
+      </c>
+      <c r="B358" t="inlineStr">
+        <is>
+          <t>mì ramen</t>
+        </is>
+      </c>
+      <c r="C358" t="inlineStr">
+        <is>
+          <t>ramen</t>
+        </is>
+      </c>
+      <c r="D358" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>banh da nem</t>
+        </is>
+      </c>
+      <c r="B359" t="inlineStr">
+        <is>
+          <t>bánh đa nem</t>
+        </is>
+      </c>
+      <c r="C359" t="inlineStr">
+        <is>
+          <t>ryzovy papir</t>
+        </is>
+      </c>
+      <c r="D359" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>mien dong</t>
+        </is>
+      </c>
+      <c r="B360" t="inlineStr">
+        <is>
+          <t>miến dong</t>
+        </is>
+      </c>
+      <c r="C360" t="inlineStr">
+        <is>
+          <t>sklenene nudle</t>
+        </is>
+      </c>
+      <c r="D360" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>bot nang</t>
+        </is>
+      </c>
+      <c r="B361" t="inlineStr">
+        <is>
+          <t>bột năng</t>
+        </is>
+      </c>
+      <c r="C361" t="inlineStr">
+        <is>
+          <t>tapiokovy skrob</t>
+        </is>
+      </c>
+      <c r="D361" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>bot gao</t>
+        </is>
+      </c>
+      <c r="B362" t="inlineStr">
+        <is>
+          <t>bột gạo</t>
+        </is>
+      </c>
+      <c r="C362" t="inlineStr">
+        <is>
+          <t>ryzova mouka</t>
+        </is>
+      </c>
+      <c r="D362" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>bot nep</t>
+        </is>
+      </c>
+      <c r="B363" t="inlineStr">
+        <is>
+          <t>bột nếp</t>
+        </is>
+      </c>
+      <c r="C363" t="inlineStr">
+        <is>
+          <t>lepkava ryzova mouka</t>
+        </is>
+      </c>
+      <c r="D363" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>tuong den</t>
+        </is>
+      </c>
+      <c r="B364" t="inlineStr">
+        <is>
+          <t>tương đen</t>
+        </is>
+      </c>
+      <c r="C364" t="inlineStr">
+        <is>
+          <t>hoisin</t>
+        </is>
+      </c>
+      <c r="D364" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>sa te</t>
+        </is>
+      </c>
+      <c r="B365" t="inlineStr">
+        <is>
+          <t>sa tế</t>
+        </is>
+      </c>
+      <c r="C365" t="inlineStr">
+        <is>
+          <t>sate</t>
+        </is>
+      </c>
+      <c r="D365" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>mam tom</t>
+        </is>
+      </c>
+      <c r="B366" t="inlineStr">
+        <is>
+          <t>mắm tôm</t>
+        </is>
+      </c>
+      <c r="C366" t="inlineStr">
+        <is>
+          <t>krevetova pasta</t>
+        </is>
+      </c>
+      <c r="D366" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>mam ruoc</t>
+        </is>
+      </c>
+      <c r="B367" t="inlineStr">
+        <is>
+          <t>mắm ruốc</t>
+        </is>
+      </c>
+      <c r="C367" t="inlineStr">
+        <is>
+          <t>krevetova pasta</t>
+        </is>
+      </c>
+      <c r="D367" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>chao</t>
+        </is>
+      </c>
+      <c r="B368" t="inlineStr">
+        <is>
+          <t>chao (đậu hũ muối)</t>
+        </is>
+      </c>
+      <c r="C368" t="inlineStr">
+        <is>
+          <t>fermentovane tofu</t>
+        </is>
+      </c>
+      <c r="D368" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>wasabi</t>
+        </is>
+      </c>
+      <c r="B369" t="inlineStr">
+        <is>
+          <t>wasabi</t>
+        </is>
+      </c>
+      <c r="C369" t="inlineStr">
+        <is>
+          <t>wasabi</t>
+        </is>
+      </c>
+      <c r="D369" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>rong bien</t>
+        </is>
+      </c>
+      <c r="B370" t="inlineStr">
+        <is>
+          <t>rong biển</t>
+        </is>
+      </c>
+      <c r="C370" t="inlineStr">
+        <is>
+          <t>morske rasy</t>
+        </is>
+      </c>
+      <c r="D370" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>la nori</t>
+        </is>
+      </c>
+      <c r="B371" t="inlineStr">
+        <is>
+          <t>lá nori</t>
+        </is>
+      </c>
+      <c r="C371" t="inlineStr">
+        <is>
+          <t>nori</t>
+        </is>
+      </c>
+      <c r="D371" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>kim chi</t>
+        </is>
+      </c>
+      <c r="B372" t="inlineStr">
+        <is>
+          <t>kim chi</t>
+        </is>
+      </c>
+      <c r="C372" t="inlineStr">
+        <is>
+          <t>kimchi</t>
+        </is>
+      </c>
+      <c r="D372" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>mang</t>
+        </is>
+      </c>
+      <c r="B373" t="inlineStr">
+        <is>
+          <t>măng</t>
+        </is>
+      </c>
+      <c r="C373" t="inlineStr">
+        <is>
+          <t>bambusove vyhonky</t>
+        </is>
+      </c>
+      <c r="D373" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>nam meo</t>
+        </is>
+      </c>
+      <c r="B374" t="inlineStr">
+        <is>
+          <t>nấm mèo</t>
+        </is>
+      </c>
+      <c r="C374" t="inlineStr">
+        <is>
+          <t>jidas usi</t>
+        </is>
+      </c>
+      <c r="D374" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>nam dong co</t>
+        </is>
+      </c>
+      <c r="B375" t="inlineStr">
+        <is>
+          <t>nấm đông cô</t>
+        </is>
+      </c>
+      <c r="C375" t="inlineStr">
+        <is>
+          <t>shiitake</t>
+        </is>
+      </c>
+      <c r="D375" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>sa</t>
+        </is>
+      </c>
+      <c r="B376" t="inlineStr">
+        <is>
+          <t>sả</t>
+        </is>
+      </c>
+      <c r="C376" t="inlineStr">
+        <is>
+          <t>citronova trava</t>
+        </is>
+      </c>
+      <c r="D376" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>la chanh</t>
+        </is>
+      </c>
+      <c r="B377" t="inlineStr">
+        <is>
+          <t>lá chanh</t>
+        </is>
+      </c>
+      <c r="C377" t="inlineStr">
+        <is>
+          <t>kaffir</t>
+        </is>
+      </c>
+      <c r="D377" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>rieng</t>
+        </is>
+      </c>
+      <c r="B378" t="inlineStr">
+        <is>
+          <t>riềng</t>
+        </is>
+      </c>
+      <c r="C378" t="inlineStr">
+        <is>
+          <t>galangal</t>
+        </is>
+      </c>
+      <c r="D378" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>nghe</t>
+        </is>
+      </c>
+      <c r="B379" t="inlineStr">
+        <is>
+          <t>nghệ</t>
+        </is>
+      </c>
+      <c r="C379" t="inlineStr">
+        <is>
+          <t>kurkuma</t>
+        </is>
+      </c>
+      <c r="D379" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>que</t>
+        </is>
+      </c>
+      <c r="B380" t="inlineStr">
+        <is>
+          <t>quế</t>
+        </is>
+      </c>
+      <c r="C380" t="inlineStr">
+        <is>
+          <t>skorice</t>
+        </is>
+      </c>
+      <c r="D380" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>hoi</t>
+        </is>
+      </c>
+      <c r="B381" t="inlineStr">
+        <is>
+          <t>hồi</t>
+        </is>
+      </c>
+      <c r="C381" t="inlineStr">
+        <is>
+          <t>badyan</t>
+        </is>
+      </c>
+      <c r="D381" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>dinh huong</t>
+        </is>
+      </c>
+      <c r="B382" t="inlineStr">
+        <is>
+          <t>đinh hương</t>
+        </is>
+      </c>
+      <c r="C382" t="inlineStr">
+        <is>
+          <t>hrebicek</t>
+        </is>
+      </c>
+      <c r="D382" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>ngu vi huong</t>
+        </is>
+      </c>
+      <c r="B383" t="inlineStr">
+        <is>
+          <t>ngũ vị hương</t>
+        </is>
+      </c>
+      <c r="C383" t="inlineStr">
+        <is>
+          <t>pet koreni</t>
+        </is>
+      </c>
+      <c r="D383" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>bot ca ri</t>
+        </is>
+      </c>
+      <c r="B384" t="inlineStr">
+        <is>
+          <t>bột cà ri</t>
+        </is>
+      </c>
+      <c r="C384" t="inlineStr">
+        <is>
+          <t>kari</t>
+        </is>
+      </c>
+      <c r="D384" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>ca ri</t>
+        </is>
+      </c>
+      <c r="B385" t="inlineStr">
+        <is>
+          <t>cà ri</t>
+        </is>
+      </c>
+      <c r="C385" t="inlineStr">
+        <is>
+          <t>kari</t>
+        </is>
+      </c>
+      <c r="D385" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>me chua</t>
+        </is>
+      </c>
+      <c r="B386" t="inlineStr">
+        <is>
+          <t>me (quả)</t>
+        </is>
+      </c>
+      <c r="C386" t="inlineStr">
+        <is>
+          <t>tamarind</t>
+        </is>
+      </c>
+      <c r="D386" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>dau do do</t>
+        </is>
+      </c>
+      <c r="B387" t="inlineStr">
+        <is>
+          <t>đậu đỏ đỗ</t>
+        </is>
+      </c>
+      <c r="C387" t="inlineStr">
+        <is>
+          <t>adzuki</t>
+        </is>
+      </c>
+      <c r="D387" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>hat sen</t>
+        </is>
+      </c>
+      <c r="B388" t="inlineStr">
+        <is>
+          <t>hạt sen</t>
+        </is>
+      </c>
+      <c r="C388" t="inlineStr">
+        <is>
+          <t>lotosova seminka</t>
+        </is>
+      </c>
+      <c r="D388" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>nuoc dua tuoi</t>
+        </is>
+      </c>
+      <c r="B389" t="inlineStr">
+        <is>
+          <t>nước dừa tươi</t>
+        </is>
+      </c>
+      <c r="C389" t="inlineStr">
+        <is>
+          <t>kokosova voda</t>
+        </is>
+      </c>
+      <c r="D389" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>sua dau nanh</t>
+        </is>
+      </c>
+      <c r="B390" t="inlineStr">
+        <is>
+          <t>sữa đậu nành</t>
+        </is>
+      </c>
+      <c r="C390" t="inlineStr">
+        <is>
+          <t>sojove mleko</t>
+        </is>
+      </c>
+      <c r="D390" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>tra sua</t>
+        </is>
+      </c>
+      <c r="B391" t="inlineStr">
+        <is>
+          <t>trà sữa</t>
+        </is>
+      </c>
+      <c r="C391" t="inlineStr">
+        <is>
+          <t>bubble tea</t>
+        </is>
+      </c>
+      <c r="D391" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>tran chau</t>
+        </is>
+      </c>
+      <c r="B392" t="inlineStr">
+        <is>
+          <t>trân châu</t>
+        </is>
+      </c>
+      <c r="C392" t="inlineStr">
+        <is>
+          <t>tapioka perly</t>
+        </is>
+      </c>
+      <c r="D392" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>gio lua</t>
+        </is>
+      </c>
+      <c r="B393" t="inlineStr">
+        <is>
+          <t>giò lụa</t>
+        </is>
+      </c>
+      <c r="C393" t="inlineStr">
+        <is>
+          <t>vietnamska sunka</t>
+        </is>
+      </c>
+      <c r="D393" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>nem chua</t>
+        </is>
+      </c>
+      <c r="B394" t="inlineStr">
+        <is>
+          <t>nem chua</t>
+        </is>
+      </c>
+      <c r="C394" t="inlineStr">
+        <is>
+          <t>nem chua</t>
+        </is>
+      </c>
+      <c r="D394" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>cha gio</t>
+        </is>
+      </c>
+      <c r="B395" t="inlineStr">
+        <is>
+          <t>chả giò</t>
+        </is>
+      </c>
+      <c r="C395" t="inlineStr">
+        <is>
+          <t>jarni zavitky</t>
+        </is>
+      </c>
+      <c r="D395" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>nem ran</t>
+        </is>
+      </c>
+      <c r="B396" t="inlineStr">
+        <is>
+          <t>nem rán</t>
+        </is>
+      </c>
+      <c r="C396" t="inlineStr">
+        <is>
+          <t>jarni zavitky</t>
+        </is>
+      </c>
+      <c r="D396" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>banh bao</t>
+        </is>
+      </c>
+      <c r="B397" t="inlineStr">
+        <is>
+          <t>bánh bao</t>
+        </is>
+      </c>
+      <c r="C397" t="inlineStr">
+        <is>
+          <t>parene knedliky</t>
+        </is>
+      </c>
+      <c r="D397" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>dim sum</t>
+        </is>
+      </c>
+      <c r="B398" t="inlineStr">
+        <is>
+          <t>dim sum</t>
+        </is>
+      </c>
+      <c r="C398" t="inlineStr">
+        <is>
+          <t>dim sum</t>
+        </is>
+      </c>
+      <c r="D398" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>dau hu chien</t>
+        </is>
+      </c>
+      <c r="B399" t="inlineStr">
+        <is>
+          <t>đậu hũ chiên</t>
+        </is>
+      </c>
+      <c r="C399" t="inlineStr">
+        <is>
+          <t>smazene tofu</t>
+        </is>
+      </c>
+      <c r="D399" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>mi a one</t>
+        </is>
+      </c>
+      <c r="B400" t="inlineStr">
+        <is>
+          <t>mì A-One</t>
+        </is>
+      </c>
+      <c r="C400" t="inlineStr">
+        <is>
+          <t>a-one</t>
+        </is>
+      </c>
+      <c r="D400" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>mi hao hao</t>
+        </is>
+      </c>
+      <c r="B401" t="inlineStr">
+        <is>
+          <t>mì Hảo Hảo</t>
+        </is>
+      </c>
+      <c r="C401" t="inlineStr">
+        <is>
+          <t>hao hao</t>
+        </is>
+      </c>
+      <c r="D401" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>mi vi phở</t>
+        </is>
+      </c>
+      <c r="B402" t="inlineStr">
+        <is>
+          <t>mì vị phở</t>
+        </is>
+      </c>
+      <c r="C402" t="inlineStr">
+        <is>
+          <t>pho nudle instantni</t>
+        </is>
+      </c>
+      <c r="D402" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>rau muong</t>
+        </is>
+      </c>
+      <c r="B403" t="inlineStr">
+        <is>
+          <t>rau muống</t>
+        </is>
+      </c>
+      <c r="C403" t="inlineStr">
+        <is>
+          <t>vodni spenat</t>
+        </is>
+      </c>
+      <c r="D403" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>cai ngot</t>
+        </is>
+      </c>
+      <c r="B404" t="inlineStr">
+        <is>
+          <t>cải ngọt</t>
+        </is>
+      </c>
+      <c r="C404" t="inlineStr">
+        <is>
+          <t>pak choi</t>
+        </is>
+      </c>
+      <c r="D404" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>cai chip</t>
+        </is>
+      </c>
+      <c r="B405" t="inlineStr">
+        <is>
+          <t>cải chíp</t>
+        </is>
+      </c>
+      <c r="C405" t="inlineStr">
+        <is>
+          <t>pak choi</t>
+        </is>
+      </c>
+      <c r="D405" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>cai be xanh</t>
+        </is>
+      </c>
+      <c r="B406" t="inlineStr">
+        <is>
+          <t>cải bẹ xanh</t>
+        </is>
+      </c>
+      <c r="C406" t="inlineStr">
+        <is>
+          <t>horcicne listy</t>
+        </is>
+      </c>
+      <c r="D406" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>su hao</t>
+        </is>
+      </c>
+      <c r="B407" t="inlineStr">
+        <is>
+          <t>su hào</t>
+        </is>
+      </c>
+      <c r="C407" t="inlineStr">
+        <is>
+          <t>kedlubna</t>
+        </is>
+      </c>
+      <c r="D407" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>su su</t>
+        </is>
+      </c>
+      <c r="B408" t="inlineStr">
+        <is>
+          <t>su su</t>
+        </is>
+      </c>
+      <c r="C408" t="inlineStr">
+        <is>
+          <t>chayote</t>
+        </is>
+      </c>
+      <c r="D408" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="409">
+      <c r="A409" t="inlineStr">
+        <is>
+          <t>dau bap</t>
+        </is>
+      </c>
+      <c r="B409" t="inlineStr">
+        <is>
+          <t>đậu bắp</t>
+        </is>
+      </c>
+      <c r="C409" t="inlineStr">
+        <is>
+          <t>okra</t>
+        </is>
+      </c>
+      <c r="D409" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="410">
+      <c r="A410" t="inlineStr">
+        <is>
+          <t>kho qua</t>
+        </is>
+      </c>
+      <c r="B410" t="inlineStr">
+        <is>
+          <t>khổ qua</t>
+        </is>
+      </c>
+      <c r="C410" t="inlineStr">
+        <is>
+          <t>horka okurka</t>
+        </is>
+      </c>
+      <c r="D410" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="411">
+      <c r="A411" t="inlineStr">
+        <is>
+          <t>muop dang</t>
+        </is>
+      </c>
+      <c r="B411" t="inlineStr">
+        <is>
+          <t>mướp đắng</t>
+        </is>
+      </c>
+      <c r="C411" t="inlineStr">
+        <is>
+          <t>horka okurka</t>
+        </is>
+      </c>
+      <c r="D411" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="412">
+      <c r="A412" t="inlineStr">
+        <is>
+          <t>khoai mon</t>
+        </is>
+      </c>
+      <c r="B412" t="inlineStr">
+        <is>
+          <t>khoai môn</t>
+        </is>
+      </c>
+      <c r="C412" t="inlineStr">
+        <is>
+          <t>taro</t>
+        </is>
+      </c>
+      <c r="D412" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="413">
+      <c r="A413" t="inlineStr">
+        <is>
+          <t>khoai mi</t>
+        </is>
+      </c>
+      <c r="B413" t="inlineStr">
+        <is>
+          <t>khoai mì</t>
+        </is>
+      </c>
+      <c r="C413" t="inlineStr">
+        <is>
+          <t>maniok</t>
+        </is>
+      </c>
+      <c r="D413" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>san</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>sắn</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>maniok</t>
+        </is>
+      </c>
+      <c r="D414" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="415">
+      <c r="A415" t="inlineStr">
+        <is>
+          <t>thit de</t>
+        </is>
+      </c>
+      <c r="B415" t="inlineStr">
+        <is>
+          <t>thịt dê</t>
+        </is>
+      </c>
+      <c r="C415" t="inlineStr">
+        <is>
+          <t>kozi maso</t>
+        </is>
+      </c>
+      <c r="D415" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="416">
+      <c r="A416" t="inlineStr">
+        <is>
+          <t>dui vit</t>
+        </is>
+      </c>
+      <c r="B416" t="inlineStr">
+        <is>
+          <t>đùi vịt</t>
+        </is>
+      </c>
+      <c r="C416" t="inlineStr">
+        <is>
+          <t>kachni stehna</t>
+        </is>
+      </c>
+      <c r="D416" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="417">
+      <c r="A417" t="inlineStr">
+        <is>
+          <t>uc vit</t>
+        </is>
+      </c>
+      <c r="B417" t="inlineStr">
+        <is>
+          <t>ức vịt</t>
+        </is>
+      </c>
+      <c r="C417" t="inlineStr">
+        <is>
+          <t>kachni prsa</t>
+        </is>
+      </c>
+      <c r="D417" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="418">
+      <c r="A418" t="inlineStr">
+        <is>
+          <t>trung vit</t>
+        </is>
+      </c>
+      <c r="B418" t="inlineStr">
+        <is>
+          <t>trứng vịt</t>
+        </is>
+      </c>
+      <c r="C418" t="inlineStr">
+        <is>
+          <t>kachni vejce</t>
+        </is>
+      </c>
+      <c r="D418" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="419">
+      <c r="A419" t="inlineStr">
+        <is>
+          <t>long ga</t>
+        </is>
+      </c>
+      <c r="B419" t="inlineStr">
+        <is>
+          <t>lòng gà</t>
+        </is>
+      </c>
+      <c r="C419" t="inlineStr">
+        <is>
+          <t>kureci drupky</t>
+        </is>
+      </c>
+      <c r="D419" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="420">
+      <c r="A420" t="inlineStr">
+        <is>
+          <t>me ga</t>
+        </is>
+      </c>
+      <c r="B420" t="inlineStr">
+        <is>
+          <t>mề gà</t>
+        </is>
+      </c>
+      <c r="C420" t="inlineStr">
+        <is>
+          <t>kureci zaludky</t>
+        </is>
+      </c>
+      <c r="D420" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="421">
+      <c r="A421" t="inlineStr">
+        <is>
+          <t>tim heo</t>
+        </is>
+      </c>
+      <c r="B421" t="inlineStr">
+        <is>
+          <t>tim heo</t>
+        </is>
+      </c>
+      <c r="C421" t="inlineStr">
+        <is>
+          <t>veprove srdce</t>
+        </is>
+      </c>
+      <c r="D421" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="422">
+      <c r="A422" t="inlineStr">
+        <is>
+          <t>long heo</t>
+        </is>
+      </c>
+      <c r="B422" t="inlineStr">
+        <is>
+          <t>lòng heo</t>
+        </is>
+      </c>
+      <c r="C422" t="inlineStr">
+        <is>
+          <t>veprove drupky</t>
+        </is>
+      </c>
+      <c r="D422" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="423">
+      <c r="A423" t="inlineStr">
+        <is>
+          <t>duoi bo</t>
+        </is>
+      </c>
+      <c r="B423" t="inlineStr">
+        <is>
+          <t>đuôi bò</t>
+        </is>
+      </c>
+      <c r="C423" t="inlineStr">
+        <is>
+          <t>hovezi ohon</t>
+        </is>
+      </c>
+      <c r="D423" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="424">
+      <c r="A424" t="inlineStr">
+        <is>
+          <t>xuong bo</t>
+        </is>
+      </c>
+      <c r="B424" t="inlineStr">
+        <is>
+          <t>xương bò</t>
+        </is>
+      </c>
+      <c r="C424" t="inlineStr">
+        <is>
+          <t>hovezi kosti</t>
+        </is>
+      </c>
+      <c r="D424" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>xuong heo</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>xương heo</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>veprove kosti</t>
+        </is>
+      </c>
+      <c r="D425" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>bap bo</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>bắp bò</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>hovezi klizka</t>
+        </is>
+      </c>
+      <c r="D426" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>luon</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>lươn</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>uhor</t>
+        </is>
+      </c>
+      <c r="D427" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>ca ro phi</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>cá rô phi</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>tilapie</t>
+        </is>
+      </c>
+      <c r="D428" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="429">
+      <c r="A429" t="inlineStr">
+        <is>
+          <t>bach tuoc</t>
+        </is>
+      </c>
+      <c r="B429" t="inlineStr">
+        <is>
+          <t>bạch tuộc</t>
+        </is>
+      </c>
+      <c r="C429" t="inlineStr">
+        <is>
+          <t>chobotnice</t>
+        </is>
+      </c>
+      <c r="D429" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="430">
+      <c r="A430" t="inlineStr">
+        <is>
+          <t>ngheu</t>
+        </is>
+      </c>
+      <c r="B430" t="inlineStr">
+        <is>
+          <t>nghêu</t>
+        </is>
+      </c>
+      <c r="C430" t="inlineStr">
+        <is>
+          <t>slavky</t>
+        </is>
+      </c>
+      <c r="D430" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="431">
+      <c r="A431" t="inlineStr">
+        <is>
+          <t>so</t>
+        </is>
+      </c>
+      <c r="B431" t="inlineStr">
+        <is>
+          <t>sò</t>
+        </is>
+      </c>
+      <c r="C431" t="inlineStr">
+        <is>
+          <t>slavky</t>
+        </is>
+      </c>
+      <c r="D431" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="432">
+      <c r="A432" t="inlineStr">
+        <is>
+          <t>hau</t>
+        </is>
+      </c>
+      <c r="B432" t="inlineStr">
+        <is>
+          <t>hàu</t>
+        </is>
+      </c>
+      <c r="C432" t="inlineStr">
+        <is>
+          <t>ustrice</t>
+        </is>
+      </c>
+      <c r="D432" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="433">
+      <c r="A433" t="inlineStr">
+        <is>
+          <t>ech</t>
+        </is>
+      </c>
+      <c r="B433" t="inlineStr">
+        <is>
+          <t>ếch</t>
+        </is>
+      </c>
+      <c r="C433" t="inlineStr">
+        <is>
+          <t>zabi stehna</t>
+        </is>
+      </c>
+      <c r="D433" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="434">
+      <c r="A434" t="inlineStr">
+        <is>
+          <t>tom su</t>
+        </is>
+      </c>
+      <c r="B434" t="inlineStr">
+        <is>
+          <t>tôm sú</t>
+        </is>
+      </c>
+      <c r="C434" t="inlineStr">
+        <is>
+          <t>tygri krevety</t>
+        </is>
+      </c>
+      <c r="D434" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="435">
+      <c r="A435" t="inlineStr">
+        <is>
+          <t>tom the</t>
+        </is>
+      </c>
+      <c r="B435" t="inlineStr">
+        <is>
+          <t>tôm thẻ</t>
+        </is>
+      </c>
+      <c r="C435" t="inlineStr">
+        <is>
+          <t>krevety vannamei</t>
+        </is>
+      </c>
+      <c r="D435" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="436">
+      <c r="A436" t="inlineStr">
+        <is>
+          <t>bia kozel</t>
+        </is>
+      </c>
+      <c r="B436" t="inlineStr">
+        <is>
+          <t>bia Kozel</t>
+        </is>
+      </c>
+      <c r="C436" t="inlineStr">
+        <is>
+          <t>kozel</t>
+        </is>
+      </c>
+      <c r="D436" t="inlineStr">
+        <is>
+          <t>Bia rượu</t>
+        </is>
+      </c>
+    </row>
+    <row r="437">
+      <c r="A437" t="inlineStr">
+        <is>
+          <t>bia pilsner</t>
+        </is>
+      </c>
+      <c r="B437" t="inlineStr">
+        <is>
+          <t>bia Pilsner</t>
+        </is>
+      </c>
+      <c r="C437" t="inlineStr">
+        <is>
+          <t>pilsner urquell</t>
+        </is>
+      </c>
+      <c r="D437" t="inlineStr">
+        <is>
+          <t>Bia rượu</t>
+        </is>
+      </c>
+    </row>
+    <row r="438">
+      <c r="A438" t="inlineStr">
+        <is>
+          <t>bia gambrinus</t>
+        </is>
+      </c>
+      <c r="B438" t="inlineStr">
+        <is>
+          <t>bia Gambrinus</t>
+        </is>
+      </c>
+      <c r="C438" t="inlineStr">
+        <is>
+          <t>gambrinus</t>
+        </is>
+      </c>
+      <c r="D438" t="inlineStr">
+        <is>
+          <t>Bia rượu</t>
+        </is>
+      </c>
+    </row>
+    <row r="439">
+      <c r="A439" t="inlineStr">
+        <is>
+          <t>bia radegast</t>
+        </is>
+      </c>
+      <c r="B439" t="inlineStr">
+        <is>
+          <t>bia Radegast</t>
+        </is>
+      </c>
+      <c r="C439" t="inlineStr">
+        <is>
+          <t>radegast</t>
+        </is>
+      </c>
+      <c r="D439" t="inlineStr">
+        <is>
+          <t>Bia rượu</t>
+        </is>
+      </c>
+    </row>
+    <row r="440">
+      <c r="A440" t="inlineStr">
+        <is>
+          <t>bia staropramen</t>
+        </is>
+      </c>
+      <c r="B440" t="inlineStr">
+        <is>
+          <t>bia Staropramen</t>
+        </is>
+      </c>
+      <c r="C440" t="inlineStr">
+        <is>
+          <t>staropramen</t>
+        </is>
+      </c>
+      <c r="D440" t="inlineStr">
+        <is>
+          <t>Bia rượu</t>
+        </is>
+      </c>
+    </row>
+    <row r="441">
+      <c r="A441" t="inlineStr">
+        <is>
+          <t>bia birell</t>
+        </is>
+      </c>
+      <c r="B441" t="inlineStr">
+        <is>
+          <t>bia Birell (không cồn)</t>
+        </is>
+      </c>
+      <c r="C441" t="inlineStr">
+        <is>
+          <t>birell</t>
+        </is>
+      </c>
+      <c r="D441" t="inlineStr">
+        <is>
+          <t>Bia rượu</t>
+        </is>
+      </c>
+    </row>
+    <row r="442">
+      <c r="A442" t="inlineStr">
+        <is>
+          <t>sua dac tatra</t>
+        </is>
+      </c>
+      <c r="B442" t="inlineStr">
+        <is>
+          <t>sữa đặc Tatra</t>
+        </is>
+      </c>
+      <c r="C442" t="inlineStr">
+        <is>
+          <t>tatra piknik</t>
+        </is>
+      </c>
+      <c r="D442" t="inlineStr">
+        <is>
+          <t>Sữa &amp; trứng</t>
+        </is>
+      </c>
+    </row>
+    <row r="443">
+      <c r="A443" t="inlineStr">
+        <is>
+          <t>pho mai parmesan</t>
+        </is>
+      </c>
+      <c r="B443" t="inlineStr">
+        <is>
+          <t>phô mai parmesan</t>
+        </is>
+      </c>
+      <c r="C443" t="inlineStr">
+        <is>
+          <t>parmezan</t>
+        </is>
+      </c>
+      <c r="D443" t="inlineStr">
+        <is>
+          <t>Sữa &amp; trứng</t>
+        </is>
+      </c>
+    </row>
+    <row r="444">
+      <c r="A444" t="inlineStr">
+        <is>
+          <t>da vien</t>
+        </is>
+      </c>
+      <c r="B444" t="inlineStr">
+        <is>
+          <t>đá viên</t>
+        </is>
+      </c>
+      <c r="C444" t="inlineStr">
+        <is>
+          <t>led</t>
+        </is>
+      </c>
+      <c r="D444" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="445">
+      <c r="A445" t="inlineStr">
+        <is>
+          <t>than nuong</t>
+        </is>
+      </c>
+      <c r="B445" t="inlineStr">
+        <is>
+          <t>than nướng</t>
+        </is>
+      </c>
+      <c r="C445" t="inlineStr">
+        <is>
+          <t>grilovaci uhli</t>
+        </is>
+      </c>
+      <c r="D445" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="446">
+      <c r="A446" t="inlineStr">
+        <is>
+          <t>giay nuong</t>
+        </is>
+      </c>
+      <c r="B446" t="inlineStr">
+        <is>
+          <t>giấy nướng</t>
+        </is>
+      </c>
+      <c r="C446" t="inlineStr">
+        <is>
+          <t>pecici papir</t>
+        </is>
+      </c>
+      <c r="D446" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="447">
+      <c r="A447" t="inlineStr">
+        <is>
+          <t>hop dung thuc an</t>
+        </is>
+      </c>
+      <c r="B447" t="inlineStr">
+        <is>
+          <t>hộp đựng thức ăn</t>
+        </is>
+      </c>
+      <c r="C447" t="inlineStr">
+        <is>
+          <t>dozy na potraviny</t>
+        </is>
+      </c>
+      <c r="D447" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v9.8: bo sung 74 tu dien tim kiem tieng Viet khong dau (446->520 muc)
Nguoi Viet khong biet tieng Sec tim de hon: rau thom (la lot, tia to,
kinh gioi...), hai san (oc, ghe, ca loc, tom kho...), rau cu (muop, bau,
mong toi, nam kim cham...), dac san Viet (nem, cha lua, banh da, mam nem,
sa te...), do kho (long nhan, ky tu, mang kho...), pho/bun. Cum nhieu tu
+ so luong van dich dung (vd "ca loc 500g" -> "hadi ryba 500g").

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tudien.xlsx
+++ b/tudien.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D447"/>
+  <dimension ref="A1:D521"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -10266,6 +10266,1634 @@
         </is>
       </c>
     </row>
+    <row r="448">
+      <c r="A448" t="inlineStr">
+        <is>
+          <t>la lot</t>
+        </is>
+      </c>
+      <c r="B448" t="inlineStr">
+        <is>
+          <t>lá lốt</t>
+        </is>
+      </c>
+      <c r="C448" t="inlineStr">
+        <is>
+          <t>piper lolot listy</t>
+        </is>
+      </c>
+      <c r="D448" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="449">
+      <c r="A449" t="inlineStr">
+        <is>
+          <t>tia to</t>
+        </is>
+      </c>
+      <c r="B449" t="inlineStr">
+        <is>
+          <t>tía tô</t>
+        </is>
+      </c>
+      <c r="C449" t="inlineStr">
+        <is>
+          <t>perilla listy</t>
+        </is>
+      </c>
+      <c r="D449" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="450">
+      <c r="A450" t="inlineStr">
+        <is>
+          <t>kinh gioi</t>
+        </is>
+      </c>
+      <c r="B450" t="inlineStr">
+        <is>
+          <t>kinh giới</t>
+        </is>
+      </c>
+      <c r="C450" t="inlineStr">
+        <is>
+          <t>vietnamska majoranka</t>
+        </is>
+      </c>
+      <c r="D450" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="451">
+      <c r="A451" t="inlineStr">
+        <is>
+          <t>hung lui</t>
+        </is>
+      </c>
+      <c r="B451" t="inlineStr">
+        <is>
+          <t>húng lủi</t>
+        </is>
+      </c>
+      <c r="C451" t="inlineStr">
+        <is>
+          <t>mata</t>
+        </is>
+      </c>
+      <c r="D451" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="452">
+      <c r="A452" t="inlineStr">
+        <is>
+          <t>bac ha</t>
+        </is>
+      </c>
+      <c r="B452" t="inlineStr">
+        <is>
+          <t>bạc hà</t>
+        </is>
+      </c>
+      <c r="C452" t="inlineStr">
+        <is>
+          <t>mata</t>
+        </is>
+      </c>
+      <c r="D452" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="453">
+      <c r="A453" t="inlineStr">
+        <is>
+          <t>rau ram</t>
+        </is>
+      </c>
+      <c r="B453" t="inlineStr">
+        <is>
+          <t>rau răm</t>
+        </is>
+      </c>
+      <c r="C453" t="inlineStr">
+        <is>
+          <t>rdesno</t>
+        </is>
+      </c>
+      <c r="D453" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="454">
+      <c r="A454" t="inlineStr">
+        <is>
+          <t>ngo gai</t>
+        </is>
+      </c>
+      <c r="B454" t="inlineStr">
+        <is>
+          <t>ngò gai</t>
+        </is>
+      </c>
+      <c r="C454" t="inlineStr">
+        <is>
+          <t>kulantro</t>
+        </is>
+      </c>
+      <c r="D454" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="455">
+      <c r="A455" t="inlineStr">
+        <is>
+          <t>thi la</t>
+        </is>
+      </c>
+      <c r="B455" t="inlineStr">
+        <is>
+          <t>thì là</t>
+        </is>
+      </c>
+      <c r="C455" t="inlineStr">
+        <is>
+          <t>kopr</t>
+        </is>
+      </c>
+      <c r="D455" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="456">
+      <c r="A456" t="inlineStr">
+        <is>
+          <t>la mo</t>
+        </is>
+      </c>
+      <c r="B456" t="inlineStr">
+        <is>
+          <t>lá mơ</t>
+        </is>
+      </c>
+      <c r="C456" t="inlineStr">
+        <is>
+          <t>paederia listy</t>
+        </is>
+      </c>
+      <c r="D456" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="457">
+      <c r="A457" t="inlineStr">
+        <is>
+          <t>la chuoi</t>
+        </is>
+      </c>
+      <c r="B457" t="inlineStr">
+        <is>
+          <t>lá chuối</t>
+        </is>
+      </c>
+      <c r="C457" t="inlineStr">
+        <is>
+          <t>bananove listy</t>
+        </is>
+      </c>
+      <c r="D457" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="458">
+      <c r="A458" t="inlineStr">
+        <is>
+          <t>hoa chuoi</t>
+        </is>
+      </c>
+      <c r="B458" t="inlineStr">
+        <is>
+          <t>hoa chuối</t>
+        </is>
+      </c>
+      <c r="C458" t="inlineStr">
+        <is>
+          <t>bananovy kvet</t>
+        </is>
+      </c>
+      <c r="D458" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="459">
+      <c r="A459" t="inlineStr">
+        <is>
+          <t>bap chuoi</t>
+        </is>
+      </c>
+      <c r="B459" t="inlineStr">
+        <is>
+          <t>bắp chuối</t>
+        </is>
+      </c>
+      <c r="C459" t="inlineStr">
+        <is>
+          <t>bananovy kvet</t>
+        </is>
+      </c>
+      <c r="D459" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="460">
+      <c r="A460" t="inlineStr">
+        <is>
+          <t>ngo sen</t>
+        </is>
+      </c>
+      <c r="B460" t="inlineStr">
+        <is>
+          <t>ngó sen</t>
+        </is>
+      </c>
+      <c r="C460" t="inlineStr">
+        <is>
+          <t>lotosove stonky</t>
+        </is>
+      </c>
+      <c r="D460" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="461">
+      <c r="A461" t="inlineStr">
+        <is>
+          <t>muop</t>
+        </is>
+      </c>
+      <c r="B461" t="inlineStr">
+        <is>
+          <t>mướp</t>
+        </is>
+      </c>
+      <c r="C461" t="inlineStr">
+        <is>
+          <t>tikev hadovita</t>
+        </is>
+      </c>
+      <c r="D461" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="462">
+      <c r="A462" t="inlineStr">
+        <is>
+          <t>muop huong</t>
+        </is>
+      </c>
+      <c r="B462" t="inlineStr">
+        <is>
+          <t>mướp hương</t>
+        </is>
+      </c>
+      <c r="C462" t="inlineStr">
+        <is>
+          <t>tikev hadovita</t>
+        </is>
+      </c>
+      <c r="D462" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="463">
+      <c r="A463" t="inlineStr">
+        <is>
+          <t>bau</t>
+        </is>
+      </c>
+      <c r="B463" t="inlineStr">
+        <is>
+          <t>bầu</t>
+        </is>
+      </c>
+      <c r="C463" t="inlineStr">
+        <is>
+          <t>tykev lahvovita</t>
+        </is>
+      </c>
+      <c r="D463" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="464">
+      <c r="A464" t="inlineStr">
+        <is>
+          <t>bi xanh</t>
+        </is>
+      </c>
+      <c r="B464" t="inlineStr">
+        <is>
+          <t>bí xanh</t>
+        </is>
+      </c>
+      <c r="C464" t="inlineStr">
+        <is>
+          <t>vinna tykev</t>
+        </is>
+      </c>
+      <c r="D464" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="465">
+      <c r="A465" t="inlineStr">
+        <is>
+          <t>bi dao</t>
+        </is>
+      </c>
+      <c r="B465" t="inlineStr">
+        <is>
+          <t>bí đao</t>
+        </is>
+      </c>
+      <c r="C465" t="inlineStr">
+        <is>
+          <t>vinna tykev</t>
+        </is>
+      </c>
+      <c r="D465" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="466">
+      <c r="A466" t="inlineStr">
+        <is>
+          <t>cai xanh</t>
+        </is>
+      </c>
+      <c r="B466" t="inlineStr">
+        <is>
+          <t>cải xanh</t>
+        </is>
+      </c>
+      <c r="C466" t="inlineStr">
+        <is>
+          <t>horcicne listy</t>
+        </is>
+      </c>
+      <c r="D466" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="467">
+      <c r="A467" t="inlineStr">
+        <is>
+          <t>cai ngong</t>
+        </is>
+      </c>
+      <c r="B467" t="inlineStr">
+        <is>
+          <t>cải ngồng</t>
+        </is>
+      </c>
+      <c r="C467" t="inlineStr">
+        <is>
+          <t>choy sum</t>
+        </is>
+      </c>
+      <c r="D467" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="468">
+      <c r="A468" t="inlineStr">
+        <is>
+          <t>mong toi</t>
+        </is>
+      </c>
+      <c r="B468" t="inlineStr">
+        <is>
+          <t>mồng tơi</t>
+        </is>
+      </c>
+      <c r="C468" t="inlineStr">
+        <is>
+          <t>malabarsky spenat</t>
+        </is>
+      </c>
+      <c r="D468" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="469">
+      <c r="A469" t="inlineStr">
+        <is>
+          <t>rau day</t>
+        </is>
+      </c>
+      <c r="B469" t="inlineStr">
+        <is>
+          <t>rau đay</t>
+        </is>
+      </c>
+      <c r="C469" t="inlineStr">
+        <is>
+          <t>jutove listy</t>
+        </is>
+      </c>
+      <c r="D469" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="470">
+      <c r="A470" t="inlineStr">
+        <is>
+          <t>rau ngot</t>
+        </is>
+      </c>
+      <c r="B470" t="inlineStr">
+        <is>
+          <t>rau ngót</t>
+        </is>
+      </c>
+      <c r="C470" t="inlineStr">
+        <is>
+          <t>sladke listy</t>
+        </is>
+      </c>
+      <c r="D470" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="471">
+      <c r="A471" t="inlineStr">
+        <is>
+          <t>rau den</t>
+        </is>
+      </c>
+      <c r="B471" t="inlineStr">
+        <is>
+          <t>rau dền</t>
+        </is>
+      </c>
+      <c r="C471" t="inlineStr">
+        <is>
+          <t>amarant listy</t>
+        </is>
+      </c>
+      <c r="D471" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="472">
+      <c r="A472" t="inlineStr">
+        <is>
+          <t>cu dau</t>
+        </is>
+      </c>
+      <c r="B472" t="inlineStr">
+        <is>
+          <t>củ đậu</t>
+        </is>
+      </c>
+      <c r="C472" t="inlineStr">
+        <is>
+          <t>jicama</t>
+        </is>
+      </c>
+      <c r="D472" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="473">
+      <c r="A473" t="inlineStr">
+        <is>
+          <t>cu sen</t>
+        </is>
+      </c>
+      <c r="B473" t="inlineStr">
+        <is>
+          <t>củ sen</t>
+        </is>
+      </c>
+      <c r="C473" t="inlineStr">
+        <is>
+          <t>lotosovy koren</t>
+        </is>
+      </c>
+      <c r="D473" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="474">
+      <c r="A474" t="inlineStr">
+        <is>
+          <t>nam rom</t>
+        </is>
+      </c>
+      <c r="B474" t="inlineStr">
+        <is>
+          <t>nấm rơm</t>
+        </is>
+      </c>
+      <c r="C474" t="inlineStr">
+        <is>
+          <t>slamova houba</t>
+        </is>
+      </c>
+      <c r="D474" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="475">
+      <c r="A475" t="inlineStr">
+        <is>
+          <t>nam kim cham</t>
+        </is>
+      </c>
+      <c r="B475" t="inlineStr">
+        <is>
+          <t>nấm kim châm</t>
+        </is>
+      </c>
+      <c r="C475" t="inlineStr">
+        <is>
+          <t>enoki</t>
+        </is>
+      </c>
+      <c r="D475" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="476">
+      <c r="A476" t="inlineStr">
+        <is>
+          <t>nam bao ngu</t>
+        </is>
+      </c>
+      <c r="B476" t="inlineStr">
+        <is>
+          <t>nấm bào ngư</t>
+        </is>
+      </c>
+      <c r="C476" t="inlineStr">
+        <is>
+          <t>hlivova houba</t>
+        </is>
+      </c>
+      <c r="D476" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="477">
+      <c r="A477" t="inlineStr">
+        <is>
+          <t>nam tuyet</t>
+        </is>
+      </c>
+      <c r="B477" t="inlineStr">
+        <is>
+          <t>nấm tuyết</t>
+        </is>
+      </c>
+      <c r="C477" t="inlineStr">
+        <is>
+          <t>bila houba</t>
+        </is>
+      </c>
+      <c r="D477" t="inlineStr">
+        <is>
+          <t>Rau củ</t>
+        </is>
+      </c>
+    </row>
+    <row r="478">
+      <c r="A478" t="inlineStr">
+        <is>
+          <t>oc</t>
+        </is>
+      </c>
+      <c r="B478" t="inlineStr">
+        <is>
+          <t>ốc</t>
+        </is>
+      </c>
+      <c r="C478" t="inlineStr">
+        <is>
+          <t>hlemyzdi</t>
+        </is>
+      </c>
+      <c r="D478" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="479">
+      <c r="A479" t="inlineStr">
+        <is>
+          <t>ghe</t>
+        </is>
+      </c>
+      <c r="B479" t="inlineStr">
+        <is>
+          <t>ghẹ</t>
+        </is>
+      </c>
+      <c r="C479" t="inlineStr">
+        <is>
+          <t>krab</t>
+        </is>
+      </c>
+      <c r="D479" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="480">
+      <c r="A480" t="inlineStr">
+        <is>
+          <t>so huyet</t>
+        </is>
+      </c>
+      <c r="B480" t="inlineStr">
+        <is>
+          <t>sò huyết</t>
+        </is>
+      </c>
+      <c r="C480" t="inlineStr">
+        <is>
+          <t>krvave mušle</t>
+        </is>
+      </c>
+      <c r="D480" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="481">
+      <c r="A481" t="inlineStr">
+        <is>
+          <t>tep</t>
+        </is>
+      </c>
+      <c r="B481" t="inlineStr">
+        <is>
+          <t>tép</t>
+        </is>
+      </c>
+      <c r="C481" t="inlineStr">
+        <is>
+          <t>male krevety</t>
+        </is>
+      </c>
+      <c r="D481" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="482">
+      <c r="A482" t="inlineStr">
+        <is>
+          <t>ca loc</t>
+        </is>
+      </c>
+      <c r="B482" t="inlineStr">
+        <is>
+          <t>cá lóc</t>
+        </is>
+      </c>
+      <c r="C482" t="inlineStr">
+        <is>
+          <t>hadi ryba</t>
+        </is>
+      </c>
+      <c r="D482" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="483">
+      <c r="A483" t="inlineStr">
+        <is>
+          <t>ca tre</t>
+        </is>
+      </c>
+      <c r="B483" t="inlineStr">
+        <is>
+          <t>cá trê</t>
+        </is>
+      </c>
+      <c r="C483" t="inlineStr">
+        <is>
+          <t>sumec</t>
+        </is>
+      </c>
+      <c r="D483" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="484">
+      <c r="A484" t="inlineStr">
+        <is>
+          <t>ca dieu hong</t>
+        </is>
+      </c>
+      <c r="B484" t="inlineStr">
+        <is>
+          <t>cá diêu hồng</t>
+        </is>
+      </c>
+      <c r="C484" t="inlineStr">
+        <is>
+          <t>tilapie cervena</t>
+        </is>
+      </c>
+      <c r="D484" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="485">
+      <c r="A485" t="inlineStr">
+        <is>
+          <t>ca keo</t>
+        </is>
+      </c>
+      <c r="B485" t="inlineStr">
+        <is>
+          <t>cá kèo</t>
+        </is>
+      </c>
+      <c r="C485" t="inlineStr">
+        <is>
+          <t>hlavacovita ryba</t>
+        </is>
+      </c>
+      <c r="D485" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="486">
+      <c r="A486" t="inlineStr">
+        <is>
+          <t>tom kho</t>
+        </is>
+      </c>
+      <c r="B486" t="inlineStr">
+        <is>
+          <t>tôm khô</t>
+        </is>
+      </c>
+      <c r="C486" t="inlineStr">
+        <is>
+          <t>susene krevety</t>
+        </is>
+      </c>
+      <c r="D486" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="487">
+      <c r="A487" t="inlineStr">
+        <is>
+          <t>muc kho</t>
+        </is>
+      </c>
+      <c r="B487" t="inlineStr">
+        <is>
+          <t>mực khô</t>
+        </is>
+      </c>
+      <c r="C487" t="inlineStr">
+        <is>
+          <t>susena olihen</t>
+        </is>
+      </c>
+      <c r="D487" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="488">
+      <c r="A488" t="inlineStr">
+        <is>
+          <t>ca kho</t>
+        </is>
+      </c>
+      <c r="B488" t="inlineStr">
+        <is>
+          <t>cá khô</t>
+        </is>
+      </c>
+      <c r="C488" t="inlineStr">
+        <is>
+          <t>susena ryba</t>
+        </is>
+      </c>
+      <c r="D488" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="489">
+      <c r="A489" t="inlineStr">
+        <is>
+          <t>thit vai</t>
+        </is>
+      </c>
+      <c r="B489" t="inlineStr">
+        <is>
+          <t>thịt vai</t>
+        </is>
+      </c>
+      <c r="C489" t="inlineStr">
+        <is>
+          <t>veprova plec</t>
+        </is>
+      </c>
+      <c r="D489" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="490">
+      <c r="A490" t="inlineStr">
+        <is>
+          <t>nam long</t>
+        </is>
+      </c>
+      <c r="B490" t="inlineStr">
+        <is>
+          <t>nạm lòng</t>
+        </is>
+      </c>
+      <c r="C490" t="inlineStr">
+        <is>
+          <t>hovezi bok</t>
+        </is>
+      </c>
+      <c r="D490" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="491">
+      <c r="A491" t="inlineStr">
+        <is>
+          <t>gan lon</t>
+        </is>
+      </c>
+      <c r="B491" t="inlineStr">
+        <is>
+          <t>gân lợn</t>
+        </is>
+      </c>
+      <c r="C491" t="inlineStr">
+        <is>
+          <t>veprove slachy</t>
+        </is>
+      </c>
+      <c r="D491" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="492">
+      <c r="A492" t="inlineStr">
+        <is>
+          <t>da lon</t>
+        </is>
+      </c>
+      <c r="B492" t="inlineStr">
+        <is>
+          <t>da lợn</t>
+        </is>
+      </c>
+      <c r="C492" t="inlineStr">
+        <is>
+          <t>veprova kuze</t>
+        </is>
+      </c>
+      <c r="D492" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="493">
+      <c r="A493" t="inlineStr">
+        <is>
+          <t>suon non</t>
+        </is>
+      </c>
+      <c r="B493" t="inlineStr">
+        <is>
+          <t>sườn non</t>
+        </is>
+      </c>
+      <c r="C493" t="inlineStr">
+        <is>
+          <t>veprova zebirka</t>
+        </is>
+      </c>
+      <c r="D493" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="494">
+      <c r="A494" t="inlineStr">
+        <is>
+          <t>mong gio</t>
+        </is>
+      </c>
+      <c r="B494" t="inlineStr">
+        <is>
+          <t>móng giò</t>
+        </is>
+      </c>
+      <c r="C494" t="inlineStr">
+        <is>
+          <t>veprove nozicky</t>
+        </is>
+      </c>
+      <c r="D494" t="inlineStr">
+        <is>
+          <t>Thịt cá</t>
+        </is>
+      </c>
+    </row>
+    <row r="495">
+      <c r="A495" t="inlineStr">
+        <is>
+          <t>nem</t>
+        </is>
+      </c>
+      <c r="B495" t="inlineStr">
+        <is>
+          <t>nem</t>
+        </is>
+      </c>
+      <c r="C495" t="inlineStr">
+        <is>
+          <t>jarni zavitky</t>
+        </is>
+      </c>
+      <c r="D495" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="496">
+      <c r="A496" t="inlineStr">
+        <is>
+          <t>cha lua</t>
+        </is>
+      </c>
+      <c r="B496" t="inlineStr">
+        <is>
+          <t>chả lụa</t>
+        </is>
+      </c>
+      <c r="C496" t="inlineStr">
+        <is>
+          <t>vietnamska sunka</t>
+        </is>
+      </c>
+      <c r="D496" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="497">
+      <c r="A497" t="inlineStr">
+        <is>
+          <t>gio cha</t>
+        </is>
+      </c>
+      <c r="B497" t="inlineStr">
+        <is>
+          <t>giò chả</t>
+        </is>
+      </c>
+      <c r="C497" t="inlineStr">
+        <is>
+          <t>vietnamska sunka</t>
+        </is>
+      </c>
+      <c r="D497" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="498">
+      <c r="A498" t="inlineStr">
+        <is>
+          <t>cha que</t>
+        </is>
+      </c>
+      <c r="B498" t="inlineStr">
+        <is>
+          <t>chả quế</t>
+        </is>
+      </c>
+      <c r="C498" t="inlineStr">
+        <is>
+          <t>skoricova sunka</t>
+        </is>
+      </c>
+      <c r="D498" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="499">
+      <c r="A499" t="inlineStr">
+        <is>
+          <t>banh da</t>
+        </is>
+      </c>
+      <c r="B499" t="inlineStr">
+        <is>
+          <t>bánh đa</t>
+        </is>
+      </c>
+      <c r="C499" t="inlineStr">
+        <is>
+          <t>ryzove chlebicky</t>
+        </is>
+      </c>
+      <c r="D499" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="500">
+      <c r="A500" t="inlineStr">
+        <is>
+          <t>banh hoi</t>
+        </is>
+      </c>
+      <c r="B500" t="inlineStr">
+        <is>
+          <t>bánh hỏi</t>
+        </is>
+      </c>
+      <c r="C500" t="inlineStr">
+        <is>
+          <t>tenke ryzove nudle</t>
+        </is>
+      </c>
+      <c r="D500" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="501">
+      <c r="A501" t="inlineStr">
+        <is>
+          <t>banh canh</t>
+        </is>
+      </c>
+      <c r="B501" t="inlineStr">
+        <is>
+          <t>bánh canh</t>
+        </is>
+      </c>
+      <c r="C501" t="inlineStr">
+        <is>
+          <t>silne ryzove nudle</t>
+        </is>
+      </c>
+      <c r="D501" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="502">
+      <c r="A502" t="inlineStr">
+        <is>
+          <t>bun tuoi</t>
+        </is>
+      </c>
+      <c r="B502" t="inlineStr">
+        <is>
+          <t>bún tươi</t>
+        </is>
+      </c>
+      <c r="C502" t="inlineStr">
+        <is>
+          <t>cerstve ryzove nudle</t>
+        </is>
+      </c>
+      <c r="D502" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="503">
+      <c r="A503" t="inlineStr">
+        <is>
+          <t>mam nem</t>
+        </is>
+      </c>
+      <c r="B503" t="inlineStr">
+        <is>
+          <t>mắm nêm</t>
+        </is>
+      </c>
+      <c r="C503" t="inlineStr">
+        <is>
+          <t>rybi pasta</t>
+        </is>
+      </c>
+      <c r="D503" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="504">
+      <c r="A504" t="inlineStr">
+        <is>
+          <t>mam tep</t>
+        </is>
+      </c>
+      <c r="B504" t="inlineStr">
+        <is>
+          <t>mắm tép</t>
+        </is>
+      </c>
+      <c r="C504" t="inlineStr">
+        <is>
+          <t>krevetova pasta</t>
+        </is>
+      </c>
+      <c r="D504" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="505">
+      <c r="A505" t="inlineStr">
+        <is>
+          <t>sa te</t>
+        </is>
+      </c>
+      <c r="B505" t="inlineStr">
+        <is>
+          <t>sa tế</t>
+        </is>
+      </c>
+      <c r="C505" t="inlineStr">
+        <is>
+          <t>sate chilli</t>
+        </is>
+      </c>
+      <c r="D505" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="506">
+      <c r="A506" t="inlineStr">
+        <is>
+          <t>tuong ban</t>
+        </is>
+      </c>
+      <c r="B506" t="inlineStr">
+        <is>
+          <t>tương bần</t>
+        </is>
+      </c>
+      <c r="C506" t="inlineStr">
+        <is>
+          <t>sojova pasta</t>
+        </is>
+      </c>
+      <c r="D506" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="507">
+      <c r="A507" t="inlineStr">
+        <is>
+          <t>dau phu ky</t>
+        </is>
+      </c>
+      <c r="B507" t="inlineStr">
+        <is>
+          <t>đậu phụ ky</t>
+        </is>
+      </c>
+      <c r="C507" t="inlineStr">
+        <is>
+          <t>susena tofu koze</t>
+        </is>
+      </c>
+      <c r="D507" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="508">
+      <c r="A508" t="inlineStr">
+        <is>
+          <t>tau hu ky</t>
+        </is>
+      </c>
+      <c r="B508" t="inlineStr">
+        <is>
+          <t>tàu hũ ky</t>
+        </is>
+      </c>
+      <c r="C508" t="inlineStr">
+        <is>
+          <t>susena tofu koze</t>
+        </is>
+      </c>
+      <c r="D508" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="509">
+      <c r="A509" t="inlineStr">
+        <is>
+          <t>long nhan</t>
+        </is>
+      </c>
+      <c r="B509" t="inlineStr">
+        <is>
+          <t>long nhãn</t>
+        </is>
+      </c>
+      <c r="C509" t="inlineStr">
+        <is>
+          <t>susene longany</t>
+        </is>
+      </c>
+      <c r="D509" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="510">
+      <c r="A510" t="inlineStr">
+        <is>
+          <t>tao tau</t>
+        </is>
+      </c>
+      <c r="B510" t="inlineStr">
+        <is>
+          <t>táo tàu</t>
+        </is>
+      </c>
+      <c r="C510" t="inlineStr">
+        <is>
+          <t>cervene datle jujube</t>
+        </is>
+      </c>
+      <c r="D510" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="511">
+      <c r="A511" t="inlineStr">
+        <is>
+          <t>ky tu</t>
+        </is>
+      </c>
+      <c r="B511" t="inlineStr">
+        <is>
+          <t>kỷ tử</t>
+        </is>
+      </c>
+      <c r="C511" t="inlineStr">
+        <is>
+          <t>goji</t>
+        </is>
+      </c>
+      <c r="D511" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="512">
+      <c r="A512" t="inlineStr">
+        <is>
+          <t>bot bang</t>
+        </is>
+      </c>
+      <c r="B512" t="inlineStr">
+        <is>
+          <t>bột báng</t>
+        </is>
+      </c>
+      <c r="C512" t="inlineStr">
+        <is>
+          <t>tapiokove kulicky</t>
+        </is>
+      </c>
+      <c r="D512" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="513">
+      <c r="A513" t="inlineStr">
+        <is>
+          <t>bot khoai</t>
+        </is>
+      </c>
+      <c r="B513" t="inlineStr">
+        <is>
+          <t>bột khoai</t>
+        </is>
+      </c>
+      <c r="C513" t="inlineStr">
+        <is>
+          <t>tapiokovy skrob</t>
+        </is>
+      </c>
+      <c r="D513" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="514">
+      <c r="A514" t="inlineStr">
+        <is>
+          <t>mang kho</t>
+        </is>
+      </c>
+      <c r="B514" t="inlineStr">
+        <is>
+          <t>măng khô</t>
+        </is>
+      </c>
+      <c r="C514" t="inlineStr">
+        <is>
+          <t>susene bambusove vyhonky</t>
+        </is>
+      </c>
+      <c r="D514" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="515">
+      <c r="A515" t="inlineStr">
+        <is>
+          <t>mang chua</t>
+        </is>
+      </c>
+      <c r="B515" t="inlineStr">
+        <is>
+          <t>măng chua</t>
+        </is>
+      </c>
+      <c r="C515" t="inlineStr">
+        <is>
+          <t>nakladane bambusove vyhonky</t>
+        </is>
+      </c>
+      <c r="D515" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="516">
+      <c r="A516" t="inlineStr">
+        <is>
+          <t>dua muoi</t>
+        </is>
+      </c>
+      <c r="B516" t="inlineStr">
+        <is>
+          <t>dưa muối</t>
+        </is>
+      </c>
+      <c r="C516" t="inlineStr">
+        <is>
+          <t>nakladana zelenina</t>
+        </is>
+      </c>
+      <c r="D516" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="517">
+      <c r="A517" t="inlineStr">
+        <is>
+          <t>ca muoi</t>
+        </is>
+      </c>
+      <c r="B517" t="inlineStr">
+        <is>
+          <t>cà muối</t>
+        </is>
+      </c>
+      <c r="C517" t="inlineStr">
+        <is>
+          <t>nakladane liliky</t>
+        </is>
+      </c>
+      <c r="D517" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="518">
+      <c r="A518" t="inlineStr">
+        <is>
+          <t>hat sen kho</t>
+        </is>
+      </c>
+      <c r="B518" t="inlineStr">
+        <is>
+          <t>hạt sen khô</t>
+        </is>
+      </c>
+      <c r="C518" t="inlineStr">
+        <is>
+          <t>susena lotosova seminka</t>
+        </is>
+      </c>
+      <c r="D518" t="inlineStr">
+        <is>
+          <t>Đồ khô &amp; gia vị</t>
+        </is>
+      </c>
+    </row>
+    <row r="519">
+      <c r="A519" t="inlineStr">
+        <is>
+          <t>pho</t>
+        </is>
+      </c>
+      <c r="B519" t="inlineStr">
+        <is>
+          <t>phở</t>
+        </is>
+      </c>
+      <c r="C519" t="inlineStr">
+        <is>
+          <t>pho ryzove nudle</t>
+        </is>
+      </c>
+      <c r="D519" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="520">
+      <c r="A520" t="inlineStr">
+        <is>
+          <t>bun bo</t>
+        </is>
+      </c>
+      <c r="B520" t="inlineStr">
+        <is>
+          <t>bún bò</t>
+        </is>
+      </c>
+      <c r="C520" t="inlineStr">
+        <is>
+          <t>hovezi pho</t>
+        </is>
+      </c>
+      <c r="D520" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
+    <row r="521">
+      <c r="A521" t="inlineStr">
+        <is>
+          <t>mien mang</t>
+        </is>
+      </c>
+      <c r="B521" t="inlineStr">
+        <is>
+          <t>miến măng</t>
+        </is>
+      </c>
+      <c r="C521" t="inlineStr">
+        <is>
+          <t>sklenene nudle</t>
+        </is>
+      </c>
+      <c r="D521" t="inlineStr">
+        <is>
+          <t>Đồ châu Á</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
v9.9: them tu dien do gia dung/bep (nerez, porcelan, talir...)
Nguoi Viet tim do bep Makro: chong ri/inox->nerez, do su->porcelan,
dia->talir, bat/to->miska, khay->podnos, ly->sklenice, dao->nuz, thot...
(520->534 muc). Cum van dich dung: "noi inox"->"hrnec nerez".

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tudien.xlsx
+++ b/tudien.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D521"/>
+  <dimension ref="A1:D535"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -11894,6 +11894,314 @@
         </is>
       </c>
     </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>chong ri</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>chống rỉ</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>nerez</t>
+        </is>
+      </c>
+      <c r="D522" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>inox</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>inox</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>nerez</t>
+        </is>
+      </c>
+      <c r="D523" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>thep khong gi</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>thép không gỉ</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>nerez</t>
+        </is>
+      </c>
+      <c r="D524" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>do su</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>đồ sứ</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>porcelan</t>
+        </is>
+      </c>
+      <c r="D525" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>bat su</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>bát sứ</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>porcelanova miska</t>
+        </is>
+      </c>
+      <c r="D526" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>dia</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>đĩa</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>talir</t>
+        </is>
+      </c>
+      <c r="D527" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>dia su</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>đĩa sứ</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>porcelanovy talir</t>
+        </is>
+      </c>
+      <c r="D528" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>bat</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>bát</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>miska</t>
+        </is>
+      </c>
+      <c r="D529" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>to</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>tô</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>miska</t>
+        </is>
+      </c>
+      <c r="D530" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>khay</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>khay</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>podnos</t>
+        </is>
+      </c>
+      <c r="D531" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>ly</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>ly</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>sklenice</t>
+        </is>
+      </c>
+      <c r="D532" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>coc</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>cốc</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>hrnek</t>
+        </is>
+      </c>
+      <c r="D533" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>dao</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>dao</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>nuz</t>
+        </is>
+      </c>
+      <c r="D534" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>thot</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>thớt</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>prkenko</t>
+        </is>
+      </c>
+      <c r="D535" t="inlineStr">
+        <is>
+          <t>Gia dụng &amp; khác</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Từ điển: thêm băng dính/keo → páska (+ 2 mặt, điện, giấy, đóng gói)
10 mục: bang dinh/bang keo/bang dan → paska; băng keo hai mặt → oboustranná
páska; băng keo điện → izolační páska; băng keo giấy → malířská páska; băng
keo đóng gói → balicí páska. dict 633 mục. v1.5.9.9.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tudien.xlsx
+++ b/tudien.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tu dien Viet-Sec" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Tu dien Viet-Sec" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D566"/>
+  <dimension ref="A1:D576"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -12884,6 +12884,226 @@
         </is>
       </c>
     </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>bang dinh</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>băng dính</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>páska</t>
+        </is>
+      </c>
+      <c r="D567" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>bang keo</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>băng keo</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>páska</t>
+        </is>
+      </c>
+      <c r="D568" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>bang dan</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>băng dán</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>páska</t>
+        </is>
+      </c>
+      <c r="D569" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>bang dinh trong</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>băng dính trong</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>lepicí páska</t>
+        </is>
+      </c>
+      <c r="D570" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>bang keo dong goi</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>băng keo đóng gói</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>balicí páska</t>
+        </is>
+      </c>
+      <c r="D571" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>bang keo hai mat</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>băng keo hai mặt</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>oboustranná páska</t>
+        </is>
+      </c>
+      <c r="D572" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>bang dinh hai mat</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>băng dính hai mặt</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>oboustranná páska</t>
+        </is>
+      </c>
+      <c r="D573" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>bang keo dien</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>băng keo điện</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>izolační páska</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>bang dinh dien</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>băng dính điện</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>izolační páska</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>bang keo giay</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>băng keo giấy</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>malířská páska</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Phân loại Akce theo danh mục chuẩn kupi.cz + 5 ô mới; bán buôn rẻ nhất trước
- Ô danh mục trước đây đoán theo chuỗi con trong tên ("cibul", "salat",
  "jahod"...) nên xếp nhầm "Bageta s cibulkou", "Kompot jahody", "Rajčata
  loupaná", "Salát s lososem" vào Rau quả. Giờ mỗi món kupi lấy breadcrumb
  chuẩn của kupi (cache kupi_cat_cache.json), món tờ rơi Tamda dùng luật
  GUESS_RULES (rau quả xét cuối cùng). retail.json thêm phần tử thứ 4.
- 5 ô mới: Rượu, Đồ hộp, Đồ khô & gia vị, Đông lạnh, Đồ ăn sẵn (10 ô cũ giữ
  nguyên thứ tự).
- Bán buôn: lấy HẾT kết quả (trước cắt 400 theo thứ tự lưu → chỉ thấy vài
  kho), xếp rẻ nhất trước theo giá/kg·lít, nút "Xem thêm" mỗi lần 40.
- Từ điển: khôi phục 34 mục (mít, vải, nhãn, băng dính...) bị routine tháng 10
  xoá khi chạy lại tao_tudien.py; script giờ tự giữ dòng sửa tay trong xlsx.
v1.6.0.16.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tudien.xlsx
+++ b/tudien.xlsx
@@ -423,7 +423,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D589"/>
+  <dimension ref="A1:D623"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -13390,6 +13390,754 @@
         </is>
       </c>
     </row>
+    <row r="590">
+      <c r="A590" t="inlineStr">
+        <is>
+          <t>trai mit</t>
+        </is>
+      </c>
+      <c r="B590" t="inlineStr">
+        <is>
+          <t>trái mít</t>
+        </is>
+      </c>
+      <c r="C590" t="inlineStr">
+        <is>
+          <t>jackfruit</t>
+        </is>
+      </c>
+      <c r="D590" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="591">
+      <c r="A591" t="inlineStr">
+        <is>
+          <t>vai</t>
+        </is>
+      </c>
+      <c r="B591" t="inlineStr">
+        <is>
+          <t>vải</t>
+        </is>
+      </c>
+      <c r="C591" t="inlineStr">
+        <is>
+          <t>lici</t>
+        </is>
+      </c>
+      <c r="D591" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="592">
+      <c r="A592" t="inlineStr">
+        <is>
+          <t>trai vai</t>
+        </is>
+      </c>
+      <c r="B592" t="inlineStr">
+        <is>
+          <t>trái vải</t>
+        </is>
+      </c>
+      <c r="C592" t="inlineStr">
+        <is>
+          <t>lici</t>
+        </is>
+      </c>
+      <c r="D592" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="593">
+      <c r="A593" t="inlineStr">
+        <is>
+          <t>trai nhan</t>
+        </is>
+      </c>
+      <c r="B593" t="inlineStr">
+        <is>
+          <t>trái nhãn</t>
+        </is>
+      </c>
+      <c r="C593" t="inlineStr">
+        <is>
+          <t>longan</t>
+        </is>
+      </c>
+      <c r="D593" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="594">
+      <c r="A594" t="inlineStr">
+        <is>
+          <t>trai oi</t>
+        </is>
+      </c>
+      <c r="B594" t="inlineStr">
+        <is>
+          <t>trái ổi</t>
+        </is>
+      </c>
+      <c r="C594" t="inlineStr">
+        <is>
+          <t>guava</t>
+        </is>
+      </c>
+      <c r="D594" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="595">
+      <c r="A595" t="inlineStr">
+        <is>
+          <t>hong</t>
+        </is>
+      </c>
+      <c r="B595" t="inlineStr">
+        <is>
+          <t>hồng</t>
+        </is>
+      </c>
+      <c r="C595" t="inlineStr">
+        <is>
+          <t>kaki</t>
+        </is>
+      </c>
+      <c r="D595" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="596">
+      <c r="A596" t="inlineStr">
+        <is>
+          <t>qua hong</t>
+        </is>
+      </c>
+      <c r="B596" t="inlineStr">
+        <is>
+          <t>quả hồng</t>
+        </is>
+      </c>
+      <c r="C596" t="inlineStr">
+        <is>
+          <t>kaki</t>
+        </is>
+      </c>
+      <c r="D596" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="597">
+      <c r="A597" t="inlineStr">
+        <is>
+          <t>khe</t>
+        </is>
+      </c>
+      <c r="B597" t="inlineStr">
+        <is>
+          <t>khế</t>
+        </is>
+      </c>
+      <c r="C597" t="inlineStr">
+        <is>
+          <t>karambola</t>
+        </is>
+      </c>
+      <c r="D597" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="598">
+      <c r="A598" t="inlineStr">
+        <is>
+          <t>trai khe</t>
+        </is>
+      </c>
+      <c r="B598" t="inlineStr">
+        <is>
+          <t>trái khế</t>
+        </is>
+      </c>
+      <c r="C598" t="inlineStr">
+        <is>
+          <t>karambola</t>
+        </is>
+      </c>
+      <c r="D598" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="599">
+      <c r="A599" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="B599" t="inlineStr">
+        <is>
+          <t>na</t>
+        </is>
+      </c>
+      <c r="C599" t="inlineStr">
+        <is>
+          <t>anona</t>
+        </is>
+      </c>
+      <c r="D599" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="600">
+      <c r="A600" t="inlineStr">
+        <is>
+          <t>mang cau</t>
+        </is>
+      </c>
+      <c r="B600" t="inlineStr">
+        <is>
+          <t>mãng cầu</t>
+        </is>
+      </c>
+      <c r="C600" t="inlineStr">
+        <is>
+          <t>anona</t>
+        </is>
+      </c>
+      <c r="D600" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="601">
+      <c r="A601" t="inlineStr">
+        <is>
+          <t>man cau</t>
+        </is>
+      </c>
+      <c r="B601" t="inlineStr">
+        <is>
+          <t>mãng cầu</t>
+        </is>
+      </c>
+      <c r="C601" t="inlineStr">
+        <is>
+          <t>anona</t>
+        </is>
+      </c>
+      <c r="D601" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="602">
+      <c r="A602" t="inlineStr">
+        <is>
+          <t>sung</t>
+        </is>
+      </c>
+      <c r="B602" t="inlineStr">
+        <is>
+          <t>sung</t>
+        </is>
+      </c>
+      <c r="C602" t="inlineStr">
+        <is>
+          <t>fiky</t>
+        </is>
+      </c>
+      <c r="D602" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="603">
+      <c r="A603" t="inlineStr">
+        <is>
+          <t>trai sung</t>
+        </is>
+      </c>
+      <c r="B603" t="inlineStr">
+        <is>
+          <t>trái sung</t>
+        </is>
+      </c>
+      <c r="C603" t="inlineStr">
+        <is>
+          <t>fiky</t>
+        </is>
+      </c>
+      <c r="D603" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="604">
+      <c r="A604" t="inlineStr">
+        <is>
+          <t>quat</t>
+        </is>
+      </c>
+      <c r="B604" t="inlineStr">
+        <is>
+          <t>quất</t>
+        </is>
+      </c>
+      <c r="C604" t="inlineStr">
+        <is>
+          <t>kumquat</t>
+        </is>
+      </c>
+      <c r="D604" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="605">
+      <c r="A605" t="inlineStr">
+        <is>
+          <t>tac</t>
+        </is>
+      </c>
+      <c r="B605" t="inlineStr">
+        <is>
+          <t>tắc</t>
+        </is>
+      </c>
+      <c r="C605" t="inlineStr">
+        <is>
+          <t>kumquat</t>
+        </is>
+      </c>
+      <c r="D605" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="606">
+      <c r="A606" t="inlineStr">
+        <is>
+          <t>du du</t>
+        </is>
+      </c>
+      <c r="B606" t="inlineStr">
+        <is>
+          <t>đu đủ</t>
+        </is>
+      </c>
+      <c r="C606" t="inlineStr">
+        <is>
+          <t>papaja</t>
+        </is>
+      </c>
+      <c r="D606" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="607">
+      <c r="A607" t="inlineStr">
+        <is>
+          <t>mo</t>
+        </is>
+      </c>
+      <c r="B607" t="inlineStr">
+        <is>
+          <t>mơ</t>
+        </is>
+      </c>
+      <c r="C607" t="inlineStr">
+        <is>
+          <t>merunky</t>
+        </is>
+      </c>
+      <c r="D607" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="608">
+      <c r="A608" t="inlineStr">
+        <is>
+          <t>cha la</t>
+        </is>
+      </c>
+      <c r="B608" t="inlineStr">
+        <is>
+          <t>chà là</t>
+        </is>
+      </c>
+      <c r="C608" t="inlineStr">
+        <is>
+          <t>datle</t>
+        </is>
+      </c>
+      <c r="D608" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="609">
+      <c r="A609" t="inlineStr">
+        <is>
+          <t>nam viet quat</t>
+        </is>
+      </c>
+      <c r="B609" t="inlineStr">
+        <is>
+          <t>nam việt quất</t>
+        </is>
+      </c>
+      <c r="C609" t="inlineStr">
+        <is>
+          <t>brusinky</t>
+        </is>
+      </c>
+      <c r="D609" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="610">
+      <c r="A610" t="inlineStr">
+        <is>
+          <t>dau</t>
+        </is>
+      </c>
+      <c r="B610" t="inlineStr">
+        <is>
+          <t>dâu</t>
+        </is>
+      </c>
+      <c r="C610" t="inlineStr">
+        <is>
+          <t>jahody</t>
+        </is>
+      </c>
+      <c r="D610" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="611">
+      <c r="A611" t="inlineStr">
+        <is>
+          <t>trai dau</t>
+        </is>
+      </c>
+      <c r="B611" t="inlineStr">
+        <is>
+          <t>trái dâu</t>
+        </is>
+      </c>
+      <c r="C611" t="inlineStr">
+        <is>
+          <t>jahody</t>
+        </is>
+      </c>
+      <c r="D611" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="612">
+      <c r="A612" t="inlineStr">
+        <is>
+          <t>dua gang</t>
+        </is>
+      </c>
+      <c r="B612" t="inlineStr">
+        <is>
+          <t>dưa gang</t>
+        </is>
+      </c>
+      <c r="C612" t="inlineStr">
+        <is>
+          <t>meloun</t>
+        </is>
+      </c>
+      <c r="D612" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="613">
+      <c r="A613" t="inlineStr">
+        <is>
+          <t>me</t>
+        </is>
+      </c>
+      <c r="B613" t="inlineStr">
+        <is>
+          <t>me</t>
+        </is>
+      </c>
+      <c r="C613" t="inlineStr">
+        <is>
+          <t>tamarind</t>
+        </is>
+      </c>
+      <c r="D613" t="inlineStr">
+        <is>
+          <t>Trái cây</t>
+        </is>
+      </c>
+    </row>
+    <row r="614">
+      <c r="A614" t="inlineStr">
+        <is>
+          <t>bang dinh</t>
+        </is>
+      </c>
+      <c r="B614" t="inlineStr">
+        <is>
+          <t>băng dính</t>
+        </is>
+      </c>
+      <c r="C614" t="inlineStr">
+        <is>
+          <t>paska</t>
+        </is>
+      </c>
+      <c r="D614" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="615">
+      <c r="A615" t="inlineStr">
+        <is>
+          <t>bang keo</t>
+        </is>
+      </c>
+      <c r="B615" t="inlineStr">
+        <is>
+          <t>băng keo</t>
+        </is>
+      </c>
+      <c r="C615" t="inlineStr">
+        <is>
+          <t>paska</t>
+        </is>
+      </c>
+      <c r="D615" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="616">
+      <c r="A616" t="inlineStr">
+        <is>
+          <t>bang dan</t>
+        </is>
+      </c>
+      <c r="B616" t="inlineStr">
+        <is>
+          <t>băng dán</t>
+        </is>
+      </c>
+      <c r="C616" t="inlineStr">
+        <is>
+          <t>paska</t>
+        </is>
+      </c>
+      <c r="D616" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="617">
+      <c r="A617" t="inlineStr">
+        <is>
+          <t>bang dinh trong</t>
+        </is>
+      </c>
+      <c r="B617" t="inlineStr">
+        <is>
+          <t>băng dính trong</t>
+        </is>
+      </c>
+      <c r="C617" t="inlineStr">
+        <is>
+          <t>lepici paska</t>
+        </is>
+      </c>
+      <c r="D617" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="618">
+      <c r="A618" t="inlineStr">
+        <is>
+          <t>bang keo dong goi</t>
+        </is>
+      </c>
+      <c r="B618" t="inlineStr">
+        <is>
+          <t>băng keo đóng gói</t>
+        </is>
+      </c>
+      <c r="C618" t="inlineStr">
+        <is>
+          <t>balici paska</t>
+        </is>
+      </c>
+      <c r="D618" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="619">
+      <c r="A619" t="inlineStr">
+        <is>
+          <t>bang keo hai mat</t>
+        </is>
+      </c>
+      <c r="B619" t="inlineStr">
+        <is>
+          <t>băng keo hai mặt</t>
+        </is>
+      </c>
+      <c r="C619" t="inlineStr">
+        <is>
+          <t>oboustranna paska</t>
+        </is>
+      </c>
+      <c r="D619" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="620">
+      <c r="A620" t="inlineStr">
+        <is>
+          <t>bang dinh hai mat</t>
+        </is>
+      </c>
+      <c r="B620" t="inlineStr">
+        <is>
+          <t>băng dính hai mặt</t>
+        </is>
+      </c>
+      <c r="C620" t="inlineStr">
+        <is>
+          <t>oboustranna paska</t>
+        </is>
+      </c>
+      <c r="D620" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="621">
+      <c r="A621" t="inlineStr">
+        <is>
+          <t>bang keo dien</t>
+        </is>
+      </c>
+      <c r="B621" t="inlineStr">
+        <is>
+          <t>băng keo điện</t>
+        </is>
+      </c>
+      <c r="C621" t="inlineStr">
+        <is>
+          <t>izolacni paska</t>
+        </is>
+      </c>
+      <c r="D621" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="622">
+      <c r="A622" t="inlineStr">
+        <is>
+          <t>bang dinh dien</t>
+        </is>
+      </c>
+      <c r="B622" t="inlineStr">
+        <is>
+          <t>băng dính điện</t>
+        </is>
+      </c>
+      <c r="C622" t="inlineStr">
+        <is>
+          <t>izolacni paska</t>
+        </is>
+      </c>
+      <c r="D622" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
+    <row r="623">
+      <c r="A623" t="inlineStr">
+        <is>
+          <t>bang keo giay</t>
+        </is>
+      </c>
+      <c r="B623" t="inlineStr">
+        <is>
+          <t>băng keo giấy</t>
+        </is>
+      </c>
+      <c r="C623" t="inlineStr">
+        <is>
+          <t>malirska paska</t>
+        </is>
+      </c>
+      <c r="D623" t="inlineStr">
+        <is>
+          <t>Văn phòng/gia dụng</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>